<commit_message>
feat(student-excel-import): luxury 3-step import UI, live data preview, department lookup, and enhanced Excel template with custom columns
</commit_message>
<xml_diff>
--- a/public/templates/students_template.xlsx
+++ b/public/templates/students_template.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="البيانات" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="بيانات الطلاب" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>الأقسام</t>
   </si>
@@ -37,7 +37,10 @@
     <t>العنوان</t>
   </si>
   <si>
-    <t>المؤهل الدراسي</t>
+    <t>الفرقة / المستوى الدراسي</t>
+  </si>
+  <si>
+    <t>الرقم السري المؤقت (اختياري)</t>
   </si>
   <si>
     <t>ملاحظات</t>
@@ -55,7 +58,7 @@
     <t>أحمد محمد علي</t>
   </si>
   <si>
-    <t>2002-05-15</t>
+    <t>2003-05-15</t>
   </si>
   <si>
     <t>ذكر</t>
@@ -67,13 +70,19 @@
     <t>+201001234567</t>
   </si>
   <si>
-    <t>ahmed@example.com</t>
+    <t>ahmed.mohamed@example.com</t>
   </si>
   <si>
     <t>القاهرة، مصر</t>
   </si>
   <si>
     <t>الفرقة الثانية</t>
+  </si>
+  <si>
+    <t>Pass@1234</t>
+  </si>
+  <si>
+    <t>طالب متفوق</t>
   </si>
   <si>
     <t/>
@@ -83,7 +92,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -91,30 +100,16 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF16A34A"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,25 +117,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF15803D"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,95 +462,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="18"/>
-  <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="18" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="20"/>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="M2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>